<commit_message>
frontend implement: component structure/layout, navbar(2)
</commit_message>
<xml_diff>
--- a/API specification.xlsx
+++ b/API specification.xlsx
@@ -19,7 +19,118 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="73">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="74">
+  <x:si>
+    <x:t>/api/semesters/{semester_id}/courses/{course_id}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/graduation</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/semesters</x:t>
+  </x:si>
+  <x:si>
+    <x:t>전공/교양 GPA 조회</x:t>
+  </x:si>
+  <x:si>
+    <x:t>학기별 이수 학점 조회</x:t>
+  </x:si>
+  <x:si>
+    <x:t>엑셀 파일 올리면 → 파싱 → semesters/courses에 자동 INSERT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/users/me/gpa/detail</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">/api/board/{post_id}/like </x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/users/me/credits</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/board/{post_id}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/graduation/status</x:t>
+  </x:si>
+  <x:si>
+    <x:t>유저 직접 수정</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/users</x:t>
+  </x:si>
+  <x:si>
+    <x:t>전체 이수 학점 조회</x:t>
+  </x:si>
+  <x:si>
+    <x:t>졸업 이수 현황 조회</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/upload</x:t>
+  </x:si>
+  <x:si>
+    <x:t>학기 목록 조회</x:t>
+  </x:si>
+  <x:si>
+    <x:t>API Path</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/board</x:t>
+  </x:si>
+  <x:si>
+    <x:t>수강 과목 목록 조회</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HTTP Method</x:t>
+  </x:si>
+  <x:si>
+    <x:t>졸업 요건 조회</x:t>
+  </x:si>
+  <x:si>
+    <x:t>학기별 GPA 조회</x:t>
+  </x:si>
+  <x:si>
+    <x:t>게시글 상세 조회</x:t>
+  </x:si>
+  <x:si>
+    <x:t>[학점·GPA]</x:t>
+  </x:si>
+  <x:si>
+    <x:t>게시글 목록 조회</x:t>
+  </x:si>
+  <x:si>
+    <x:t>졸업 기준 설정</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/users/</x:t>
+  </x:si>
+  <x:si>
+    <x:t>누적 GPA 조회</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/board/{post_id}/comments</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">/api/board/{post_id}/bookmark </x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/semesters/{semester_id}</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">/api/board/{post_id}/comments </x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/graduation/requirements</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/semesters/{semester_id}/gpa</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/board/{post_id}/comments/{id}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/users/login</x:t>
+  </x:si>
   <x:si>
     <x:t>/api/users/mypage</x:t>
   </x:si>
@@ -27,217 +138,109 @@
     <x:t>/api/users/me/gpa</x:t>
   </x:si>
   <x:si>
-    <x:t>/api/users/login</x:t>
+    <x:t>POST</x:t>
+  </x:si>
+  <x:si>
+    <x:t>개발O 통합X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>index</x:t>
+  </x:si>
+  <x:si>
+    <x:t>개발 현황</x:t>
+  </x:si>
+  <x:si>
+    <x:t>게시글 작성</x:t>
+  </x:si>
+  <x:si>
+    <x:t>[회원]</x:t>
+  </x:si>
+  <x:si>
+    <x:t>과목 삭제</x:t>
+  </x:si>
+  <x:si>
+    <x:t>과목 추가</x:t>
+  </x:si>
+  <x:si>
+    <x:t>학기 추가</x:t>
+  </x:si>
+  <x:si>
+    <x:t>게시글 수정</x:t>
+  </x:si>
+  <x:si>
+    <x:t>[학기]</x:t>
+  </x:si>
+  <x:si>
+    <x:t>[졸업 요건]</x:t>
+  </x:si>
+  <x:si>
+    <x:t>게시글 삭제</x:t>
+  </x:si>
+  <x:si>
+    <x:t>회원 탈퇴</x:t>
+  </x:si>
+  <x:si>
+    <x:t>댓글 작성</x:t>
+  </x:si>
+  <x:si>
+    <x:t>API 명세서</x:t>
+  </x:si>
+  <x:si>
+    <x:t>과목 수정</x:t>
+  </x:si>
+  <x:si>
+    <x:t>[과목]</x:t>
+  </x:si>
+  <x:si>
+    <x:t>회원가입</x:t>
+  </x:si>
+  <x:si>
+    <x:t>학기 삭제</x:t>
+  </x:si>
+  <x:si>
+    <x:t>댓글 삭제</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DELETE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>댓글 목록</x:t>
+  </x:si>
+  <x:si>
+    <x:t>[게시판]</x:t>
+  </x:si>
+  <x:si>
+    <x:t>내 정보 조회</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/semesters/{semester_id}/credits</x:t>
+  </x:si>
+  <x:si>
+    <x:t>/api/semesters/{semester_id}/courses</x:t>
   </x:si>
   <x:si>
     <x:t>북마크</x:t>
   </x:si>
   <x:si>
-    <x:t>학기별 이수 학점 조회</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/graduation</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/semesters</x:t>
-  </x:si>
-  <x:si>
-    <x:t>전공/교양 GPA 조회</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/semesters/{semester_id}/courses/{course_id}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HTTP Method</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/users</x:t>
-  </x:si>
-  <x:si>
-    <x:t>수강 과목 목록 조회</x:t>
-  </x:si>
-  <x:si>
-    <x:t>API Path</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/users/</x:t>
-  </x:si>
-  <x:si>
-    <x:t>학기 목록 조회</x:t>
-  </x:si>
-  <x:si>
-    <x:t>누적 GPA 조회</x:t>
-  </x:si>
-  <x:si>
-    <x:t>전체 이수 학점 조회</x:t>
-  </x:si>
-  <x:si>
-    <x:t>졸업 이수 현황 조회</x:t>
-  </x:si>
-  <x:si>
-    <x:t>[학점·GPA]</x:t>
-  </x:si>
-  <x:si>
-    <x:t>학기별 GPA 조회</x:t>
-  </x:si>
-  <x:si>
-    <x:t>졸업 요건 조회</x:t>
-  </x:si>
-  <x:si>
-    <x:t>졸업 기준 설정</x:t>
+    <x:t>기능</x:t>
+  </x:si>
+  <x:si>
+    <x:t>로그인</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PUT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>메모</x:t>
   </x:si>
   <x:si>
     <x:t>좋아요</x:t>
   </x:si>
   <x:si>
-    <x:t>엑셀 파일 올리면 → 파싱 → semesters/courses에 자동 INSERT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/users/me/gpa/detail</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/semesters/{semester_id}/gpa</x:t>
-  </x:si>
-  <x:si>
-    <x:t>게시글 목록 조회</x:t>
-  </x:si>
-  <x:si>
-    <x:t>게시글 상세 조회</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/board</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/semesters/{semester_id}/courses</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/semesters/{semester_id}/credits</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기능</x:t>
-  </x:si>
-  <x:si>
-    <x:t>로그인</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PUT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>[학기]</x:t>
-  </x:si>
-  <x:si>
-    <x:t>학기 추가</x:t>
-  </x:si>
-  <x:si>
-    <x:t>과목 추가</x:t>
-  </x:si>
-  <x:si>
-    <x:t>[회원]</x:t>
-  </x:si>
-  <x:si>
-    <x:t>POST</x:t>
-  </x:si>
-  <x:si>
-    <x:t>과목 수정</x:t>
-  </x:si>
-  <x:si>
-    <x:t>[게시판]</x:t>
-  </x:si>
-  <x:si>
-    <x:t>게시글 작성</x:t>
-  </x:si>
-  <x:si>
-    <x:t>게시글 수정</x:t>
-  </x:si>
-  <x:si>
-    <x:t>index</x:t>
-  </x:si>
-  <x:si>
-    <x:t>[과목]</x:t>
-  </x:si>
-  <x:si>
-    <x:t>[졸업 요건]</x:t>
-  </x:si>
-  <x:si>
-    <x:t>내 정보 조회</x:t>
-  </x:si>
-  <x:si>
-    <x:t>게시글 삭제</x:t>
-  </x:si>
-  <x:si>
-    <x:t>개발 현황</x:t>
-  </x:si>
-  <x:si>
-    <x:t>과목 삭제</x:t>
-  </x:si>
-  <x:si>
-    <x:t>API 명세서</x:t>
-  </x:si>
-  <x:si>
-    <x:t>회원가입</x:t>
-  </x:si>
-  <x:si>
-    <x:t>회원 탈퇴</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DELETE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>학기 삭제</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/semesters/{semester_id}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/graduation/requirements</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/users/me/credits</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/graduation/status</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/board/{post_id}</x:t>
-  </x:si>
-  <x:si>
     <x:t>비고</x:t>
-  </x:si>
-  <x:si>
-    <x:t>댓글 삭제</x:t>
-  </x:si>
-  <x:si>
-    <x:t>댓글 작성</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/api/board/{post_id}/comments </x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/upload</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/api/board/{post_id}/like </x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/api/board/{post_id}/bookmark </x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/board/{post_id}/comments</x:t>
-  </x:si>
-  <x:si>
-    <x:t>댓글 목록</x:t>
-  </x:si>
-  <x:si>
-    <x:t>메모</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/api/board/{post_id}/comments/{id}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>유저 직접 수정</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -276,6 +279,11 @@
       <x:color rgb="ff000000"/>
     </x:font>
     <x:font>
+      <x:name val="맑은 고딕"/>
+      <x:sz val="11"/>
+      <x:color rgb="ff000000"/>
+    </x:font>
+    <x:font>
       <x:name val="&quot;맑은 고딕&quot;"/>
       <x:sz val="10"/>
       <x:color rgb="ff000000"/>
@@ -287,48 +295,17 @@
       <x:color rgb="ff444444"/>
       <x:i val="1"/>
     </x:font>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
-        <x:font hs:extension="1">
-          <x:name val="&quot;맑은 고딕&quot;"/>
-          <x:sz val="10"/>
-          <x:color rgb="ff000000"/>
-          <hs:size val="100"/>
-          <hs:ratio val="100"/>
-          <hs:spacing val="0"/>
-          <hs:offset val="0"/>
-        </x:font>
-      </mc:Choice>
-      <mc:Fallback>
-        <x:font>
-          <x:name val="&quot;맑은 고딕&quot;"/>
-          <x:sz val="10"/>
-          <x:color rgb="ff000000"/>
-        </x:font>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
-        <x:font hs:extension="1">
-          <x:name val="&quot;맑은 고딕&quot;"/>
-          <x:sz val="9"/>
-          <x:color rgb="ff1a5c38"/>
-          <x:b val="1"/>
-          <hs:size val="100"/>
-          <hs:ratio val="100"/>
-          <hs:spacing val="0"/>
-          <hs:offset val="0"/>
-        </x:font>
-      </mc:Choice>
-      <mc:Fallback>
-        <x:font>
-          <x:name val="&quot;맑은 고딕&quot;"/>
-          <x:sz val="9"/>
-          <x:color rgb="ff1a5c38"/>
-          <x:b val="1"/>
-        </x:font>
-      </mc:Fallback>
-    </mc:AlternateContent>
+    <x:font>
+      <x:name val="&quot;맑은 고딕&quot;"/>
+      <x:sz val="10"/>
+      <x:color rgb="ff000000"/>
+    </x:font>
+    <x:font>
+      <x:name val="&quot;맑은 고딕&quot;"/>
+      <x:sz val="9"/>
+      <x:color rgb="ff1a5c38"/>
+      <x:b val="1"/>
+    </x:font>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
         <x:font hs:extension="1">
@@ -479,23 +456,6 @@
         </x:font>
       </mc:Fallback>
     </mc:AlternateContent>
-    <x:font>
-      <x:name val="&quot;맑은 고딕&quot;"/>
-      <x:sz val="16"/>
-      <x:color rgb="ff000000"/>
-      <x:b val="1"/>
-    </x:font>
-    <x:font>
-      <x:name val="&quot;맑은 고딕&quot;"/>
-      <x:sz val="10"/>
-      <x:color rgb="ff2b4590"/>
-      <x:b val="1"/>
-    </x:font>
-    <x:font>
-      <x:name val="맑은 고딕"/>
-      <x:sz val="11"/>
-      <x:color rgb="ff000000"/>
-    </x:font>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
         <x:font hs:extension="1">
@@ -537,6 +497,50 @@
           <x:sz val="11"/>
           <x:color rgb="ff000000"/>
           <x:i val="1"/>
+        </x:font>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:font hs:extension="1">
+          <x:name val="&quot;맑은 고딕&quot;"/>
+          <x:sz val="16"/>
+          <x:color rgb="ff000000"/>
+          <x:b val="1"/>
+          <hs:size val="100"/>
+          <hs:ratio val="100"/>
+          <hs:spacing val="0"/>
+          <hs:offset val="0"/>
+        </x:font>
+      </mc:Choice>
+      <mc:Fallback>
+        <x:font>
+          <x:name val="&quot;맑은 고딕&quot;"/>
+          <x:sz val="16"/>
+          <x:color rgb="ff000000"/>
+          <x:b val="1"/>
+        </x:font>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:font hs:extension="1">
+          <x:name val="&quot;맑은 고딕&quot;"/>
+          <x:sz val="10"/>
+          <x:color rgb="ff2b4590"/>
+          <x:b val="1"/>
+          <hs:size val="100"/>
+          <hs:ratio val="100"/>
+          <hs:spacing val="0"/>
+          <hs:offset val="0"/>
+        </x:font>
+      </mc:Choice>
+      <mc:Fallback>
+        <x:font>
+          <x:name val="&quot;맑은 고딕&quot;"/>
+          <x:sz val="10"/>
+          <x:color rgb="ff2b4590"/>
+          <x:b val="1"/>
         </x:font>
       </mc:Fallback>
     </mc:AlternateContent>
@@ -634,7 +638,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="19" fillId="0" borderId="0">
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
@@ -644,136 +648,148 @@
     </x:xf>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
-        <x:xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
+        <x:xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
           <x:alignment horizontal="center" vertical="bottom"/>
           <hs:parashape hs:lineSpacingType="betweenLines" hs:lineSpacing="75" hs:breakNonLatinWord="breakWord" hs:breakLatinWord="keepWord" hs:condense="0" hs:textAlignment="baseLine"/>
         </x:xf>
       </mc:Choice>
       <mc:Fallback>
-        <x:xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-          <x:alignment horizontal="center" vertical="bottom"/>
-        </x:xf>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
-        <x:xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
+        <x:xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+          <x:alignment horizontal="center" vertical="bottom"/>
+        </x:xf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
           <x:alignment horizontal="center" vertical="bottom"/>
           <hs:parashape hs:lineSpacingType="betweenLines" hs:lineSpacing="75" hs:breakNonLatinWord="breakWord" hs:breakLatinWord="keepWord" hs:condense="0" hs:textAlignment="baseLine"/>
         </x:xf>
       </mc:Choice>
       <mc:Fallback>
-        <x:xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-          <x:alignment horizontal="center" vertical="bottom"/>
-        </x:xf>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <x:xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+        <x:xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+          <x:alignment horizontal="center" vertical="bottom"/>
+        </x:xf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="bottom"/>
     </x:xf>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
-        <x:xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
+        <x:xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
           <x:alignment horizontal="center" vertical="bottom"/>
           <hs:parashape hs:lineSpacingType="betweenLines" hs:lineSpacing="75" hs:breakNonLatinWord="breakWord" hs:breakLatinWord="keepWord" hs:condense="0" hs:textAlignment="baseLine"/>
         </x:xf>
       </mc:Choice>
       <mc:Fallback>
-        <x:xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-          <x:alignment horizontal="center" vertical="bottom"/>
-        </x:xf>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <x:xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+        <x:xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+          <x:alignment horizontal="center" vertical="bottom"/>
+        </x:xf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="bottom"/>
     </x:xf>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
-        <x:xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
+        <x:xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
           <x:alignment horizontal="center" vertical="bottom"/>
           <hs:parashape hs:lineSpacingType="betweenLines" hs:lineSpacing="75" hs:breakNonLatinWord="breakWord" hs:breakLatinWord="keepWord" hs:condense="0" hs:textAlignment="baseLine"/>
         </x:xf>
       </mc:Choice>
       <mc:Fallback>
-        <x:xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-          <x:alignment horizontal="center" vertical="bottom"/>
-        </x:xf>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
-        <x:xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
+        <x:xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+          <x:alignment horizontal="center" vertical="bottom"/>
+        </x:xf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
           <x:alignment horizontal="center" vertical="bottom"/>
           <hs:parashape hs:lineSpacingType="betweenLines" hs:lineSpacing="75" hs:breakNonLatinWord="breakWord" hs:breakLatinWord="keepWord" hs:condense="0" hs:textAlignment="baseLine"/>
         </x:xf>
       </mc:Choice>
       <mc:Fallback>
-        <x:xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-          <x:alignment horizontal="center" vertical="bottom"/>
-        </x:xf>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
-        <x:xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
+        <x:xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+          <x:alignment horizontal="center" vertical="bottom"/>
+        </x:xf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
           <x:alignment horizontal="center" vertical="bottom"/>
           <hs:parashape hs:lineSpacingType="betweenLines" hs:lineSpacing="75" hs:breakNonLatinWord="breakWord" hs:breakLatinWord="keepWord" hs:condense="0" hs:textAlignment="baseLine"/>
         </x:xf>
       </mc:Choice>
       <mc:Fallback>
-        <x:xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-          <x:alignment horizontal="center" vertical="bottom"/>
-        </x:xf>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
-        <x:xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
+        <x:xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+          <x:alignment horizontal="center" vertical="bottom"/>
+        </x:xf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
           <x:alignment horizontal="center" vertical="bottom"/>
           <hs:parashape hs:lineSpacingType="betweenLines" hs:lineSpacing="75" hs:breakNonLatinWord="breakWord" hs:breakLatinWord="keepWord" hs:condense="0" hs:textAlignment="baseLine"/>
         </x:xf>
       </mc:Choice>
       <mc:Fallback>
-        <x:xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-          <x:alignment horizontal="center" vertical="bottom"/>
-        </x:xf>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
-        <x:xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
+        <x:xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+          <x:alignment horizontal="center" vertical="bottom"/>
+        </x:xf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
           <x:alignment horizontal="center" vertical="bottom"/>
           <hs:parashape hs:lineSpacingType="betweenLines" hs:lineSpacing="75" hs:breakNonLatinWord="breakWord" hs:breakLatinWord="keepWord" hs:condense="0" hs:textAlignment="baseLine"/>
         </x:xf>
       </mc:Choice>
       <mc:Fallback>
-        <x:xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-          <x:alignment horizontal="center" vertical="bottom"/>
-        </x:xf>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
-        <x:xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
+        <x:xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+          <x:alignment horizontal="center" vertical="bottom"/>
+        </x:xf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
           <x:alignment horizontal="center" vertical="bottom"/>
           <hs:parashape hs:lineSpacingType="betweenLines" hs:lineSpacing="75" hs:breakNonLatinWord="breakWord" hs:breakLatinWord="keepWord" hs:condense="0" hs:textAlignment="baseLine"/>
         </x:xf>
       </mc:Choice>
       <mc:Fallback>
-        <x:xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-          <x:alignment horizontal="center" vertical="bottom"/>
-        </x:xf>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
-        <x:xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
+        <x:xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+          <x:alignment horizontal="center" vertical="bottom"/>
+        </x:xf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="center"/>
+    </x:xf>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:xf numFmtId="0" fontId="20" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" hs:applyExtension="1">
           <x:alignment horizontal="center" vertical="bottom"/>
           <hs:parashape hs:lineSpacingType="betweenLines" hs:lineSpacing="75" hs:breakNonLatinWord="breakWord" hs:breakLatinWord="keepWord" hs:condense="0" hs:textAlignment="baseLine"/>
         </x:xf>
       </mc:Choice>
       <mc:Fallback>
-        <x:xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+        <x:xf numFmtId="0" fontId="20" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
           <x:alignment horizontal="center" vertical="bottom"/>
         </x:xf>
       </mc:Fallback>
@@ -784,31 +800,19 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="21" fillId="2" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="bottom"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="center"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
-    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="3">
     <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <x:cellStyle name="표준" xfId="2" builtinId="0" iLevel="0"/>
+    <x:cellStyle name="표준" xfId="2"/>
   </x:cellStyles>
   <x:dxfs count="1">
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -1051,66 +1055,66 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:9" ht="28.5" customHeight="1">
-      <x:c r="A1" s="12" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="B1" s="13"/>
-      <x:c r="C1" s="13"/>
-      <x:c r="D1" s="13"/>
-      <x:c r="E1" s="13"/>
-      <x:c r="F1" s="13"/>
-      <x:c r="G1" s="13"/>
-      <x:c r="H1" s="13"/>
-      <x:c r="I1" s="14"/>
+      <x:c r="A1" s="16" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B1" s="17"/>
+      <x:c r="C1" s="17"/>
+      <x:c r="D1" s="17"/>
+      <x:c r="E1" s="17"/>
+      <x:c r="F1" s="17"/>
+      <x:c r="G1" s="17"/>
+      <x:c r="H1" s="17"/>
+      <x:c r="I1" s="18"/>
     </x:row>
     <x:row r="2" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A2" s="1" t="s">
-        <x:v>44</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>9</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
-        <x:v>49</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G2" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="H2" s="1"/>
       <x:c r="I2" s="1"/>
     </x:row>
     <x:row r="3" spans="1:9" ht="13.19999999999999928946">
-      <x:c r="A3" s="15" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="B3" s="13"/>
-      <x:c r="C3" s="13"/>
-      <x:c r="D3" s="13"/>
-      <x:c r="E3" s="13"/>
-      <x:c r="F3" s="13"/>
-      <x:c r="G3" s="13"/>
-      <x:c r="H3" s="13"/>
-      <x:c r="I3" s="14"/>
+      <x:c r="A3" s="19" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B3" s="17"/>
+      <x:c r="C3" s="17"/>
+      <x:c r="D3" s="17"/>
+      <x:c r="E3" s="17"/>
+      <x:c r="F3" s="17"/>
+      <x:c r="G3" s="17"/>
+      <x:c r="H3" s="17"/>
+      <x:c r="I3" s="18"/>
     </x:row>
     <x:row r="4" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A4" s="2"/>
       <x:c r="B4" s="3" t="s">
-        <x:v>52</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C4" s="4" t="s">
         <x:v>39</x:v>
       </x:c>
       <x:c r="D4" s="5" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E4" s="6"/>
       <x:c r="F4" s="7"/>
@@ -1121,13 +1125,13 @@
     <x:row r="5" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A5" s="2"/>
       <x:c r="B5" s="3" t="s">
-        <x:v>33</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C5" s="4" t="s">
         <x:v>39</x:v>
       </x:c>
       <x:c r="D5" s="5" t="s">
-        <x:v>2</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E5" s="6"/>
       <x:c r="F5" s="7"/>
@@ -1138,13 +1142,13 @@
     <x:row r="6" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A6" s="2"/>
       <x:c r="B6" s="3" t="s">
-        <x:v>47</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C6" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D6" s="5" t="s">
-        <x:v>0</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E6" s="6"/>
       <x:c r="F6" s="7"/>
@@ -1155,13 +1159,13 @@
     <x:row r="7" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A7" s="2"/>
       <x:c r="B7" s="3" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C7" s="10" t="s">
-        <x:v>54</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D7" s="5" t="s">
-        <x:v>13</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E7" s="6"/>
       <x:c r="F7" s="7"/>
@@ -1170,28 +1174,28 @@
       <x:c r="I7" s="7"/>
     </x:row>
     <x:row r="8" spans="1:9" ht="13.19999999999999928946">
-      <x:c r="A8" s="15" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="B8" s="13"/>
-      <x:c r="C8" s="13"/>
-      <x:c r="D8" s="13"/>
-      <x:c r="E8" s="13"/>
-      <x:c r="F8" s="13"/>
-      <x:c r="G8" s="13"/>
-      <x:c r="H8" s="13"/>
-      <x:c r="I8" s="14"/>
+      <x:c r="A8" s="19" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B8" s="17"/>
+      <x:c r="C8" s="17"/>
+      <x:c r="D8" s="17"/>
+      <x:c r="E8" s="17"/>
+      <x:c r="F8" s="17"/>
+      <x:c r="G8" s="17"/>
+      <x:c r="H8" s="17"/>
+      <x:c r="I8" s="18"/>
     </x:row>
     <x:row r="9" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A9" s="2"/>
       <x:c r="B9" s="3" t="s">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C9" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D9" s="5" t="s">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E9" s="6"/>
       <x:c r="F9" s="7"/>
@@ -1202,16 +1206,16 @@
     <x:row r="10" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A10" s="2"/>
       <x:c r="B10" s="3" t="s">
-        <x:v>36</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C10" s="4" t="s">
         <x:v>39</x:v>
       </x:c>
       <x:c r="D10" s="5" t="s">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E10" s="6" t="s">
-        <x:v>72</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F10" s="7"/>
       <x:c r="G10" s="8"/>
@@ -1221,13 +1225,13 @@
     <x:row r="11" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A11" s="2"/>
       <x:c r="B11" s="3" t="s">
-        <x:v>55</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C11" s="10" t="s">
-        <x:v>54</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D11" s="5" t="s">
-        <x:v>56</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E11" s="6"/>
       <x:c r="F11" s="7"/>
@@ -1236,28 +1240,28 @@
       <x:c r="I11" s="7"/>
     </x:row>
     <x:row r="12" spans="1:9" ht="13.19999999999999928946">
-      <x:c r="A12" s="15" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="B12" s="13"/>
-      <x:c r="C12" s="13"/>
-      <x:c r="D12" s="13"/>
-      <x:c r="E12" s="13"/>
-      <x:c r="F12" s="13"/>
-      <x:c r="G12" s="13"/>
-      <x:c r="H12" s="13"/>
-      <x:c r="I12" s="14"/>
+      <x:c r="A12" s="19" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B12" s="17"/>
+      <x:c r="C12" s="17"/>
+      <x:c r="D12" s="17"/>
+      <x:c r="E12" s="17"/>
+      <x:c r="F12" s="17"/>
+      <x:c r="G12" s="17"/>
+      <x:c r="H12" s="17"/>
+      <x:c r="I12" s="18"/>
     </x:row>
     <x:row r="13" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A13" s="2"/>
       <x:c r="B13" s="3" t="s">
-        <x:v>11</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C13" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D13" s="5" t="s">
-        <x:v>29</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E13" s="6"/>
       <x:c r="F13" s="7"/>
@@ -1268,13 +1272,13 @@
     <x:row r="14" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A14" s="2"/>
       <x:c r="B14" s="3" t="s">
-        <x:v>37</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C14" s="4" t="s">
         <x:v>39</x:v>
       </x:c>
       <x:c r="D14" s="5" t="s">
-        <x:v>29</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E14" s="6"/>
       <x:c r="F14" s="7"/>
@@ -1285,13 +1289,13 @@
     <x:row r="15" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A15" s="2"/>
       <x:c r="B15" s="3" t="s">
-        <x:v>40</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C15" s="11" t="s">
-        <x:v>34</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="D15" s="5" t="s">
-        <x:v>8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E15" s="6"/>
       <x:c r="F15" s="7"/>
@@ -1302,13 +1306,13 @@
     <x:row r="16" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A16" s="2"/>
       <x:c r="B16" s="3" t="s">
-        <x:v>50</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C16" s="10" t="s">
-        <x:v>54</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D16" s="5" t="s">
-        <x:v>8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E16" s="6"/>
       <x:c r="F16" s="7"/>
@@ -1317,28 +1321,28 @@
       <x:c r="I16" s="7"/>
     </x:row>
     <x:row r="17" spans="1:9" ht="13.19999999999999928946">
-      <x:c r="A17" s="15" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B17" s="13"/>
-      <x:c r="C17" s="13"/>
-      <x:c r="D17" s="13"/>
-      <x:c r="E17" s="13"/>
-      <x:c r="F17" s="13"/>
-      <x:c r="G17" s="13"/>
-      <x:c r="H17" s="13"/>
-      <x:c r="I17" s="14"/>
+      <x:c r="A17" s="19" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B17" s="17"/>
+      <x:c r="C17" s="17"/>
+      <x:c r="D17" s="17"/>
+      <x:c r="E17" s="17"/>
+      <x:c r="F17" s="17"/>
+      <x:c r="G17" s="17"/>
+      <x:c r="H17" s="17"/>
+      <x:c r="I17" s="18"/>
     </x:row>
     <x:row r="18" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A18" s="2"/>
       <x:c r="B18" s="3" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C18" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D18" s="5" t="s">
-        <x:v>25</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E18" s="6"/>
       <x:c r="F18" s="7"/>
@@ -1349,13 +1353,13 @@
     <x:row r="19" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A19" s="2"/>
       <x:c r="B19" s="3" t="s">
-        <x:v>15</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C19" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D19" s="5" t="s">
-        <x:v>1</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E19" s="6"/>
       <x:c r="F19" s="7"/>
@@ -1366,13 +1370,13 @@
     <x:row r="20" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A20" s="2"/>
       <x:c r="B20" s="3" t="s">
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C20" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D20" s="5" t="s">
-        <x:v>24</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E20" s="6"/>
       <x:c r="F20" s="7"/>
@@ -1386,10 +1390,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C21" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D21" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E21" s="6"/>
       <x:c r="F21" s="7"/>
@@ -1400,13 +1404,13 @@
     <x:row r="22" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A22" s="2"/>
       <x:c r="B22" s="3" t="s">
-        <x:v>16</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C22" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D22" s="5" t="s">
-        <x:v>58</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E22" s="6"/>
       <x:c r="F22" s="7"/>
@@ -1415,28 +1419,28 @@
       <x:c r="I22" s="7"/>
     </x:row>
     <x:row r="23" spans="1:9" ht="13.19999999999999928946">
-      <x:c r="A23" s="15" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="B23" s="13"/>
-      <x:c r="C23" s="13"/>
-      <x:c r="D23" s="13"/>
-      <x:c r="E23" s="13"/>
-      <x:c r="F23" s="13"/>
-      <x:c r="G23" s="13"/>
-      <x:c r="H23" s="13"/>
-      <x:c r="I23" s="14"/>
+      <x:c r="A23" s="19" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B23" s="17"/>
+      <x:c r="C23" s="17"/>
+      <x:c r="D23" s="17"/>
+      <x:c r="E23" s="17"/>
+      <x:c r="F23" s="17"/>
+      <x:c r="G23" s="17"/>
+      <x:c r="H23" s="17"/>
+      <x:c r="I23" s="18"/>
     </x:row>
     <x:row r="24" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A24" s="2"/>
       <x:c r="B24" s="3" t="s">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C24" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D24" s="5" t="s">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E24" s="6"/>
       <x:c r="F24" s="7"/>
@@ -1447,13 +1451,13 @@
     <x:row r="25" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A25" s="2"/>
       <x:c r="B25" s="3" t="s">
-        <x:v>17</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C25" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D25" s="5" t="s">
-        <x:v>59</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E25" s="6"/>
       <x:c r="F25" s="7"/>
@@ -1464,45 +1468,45 @@
     <x:row r="26" spans="1:9" ht="13.19999999999999928946">
       <x:c r="A26" s="2"/>
       <x:c r="B26" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C26" s="4" t="s">
         <x:v>39</x:v>
       </x:c>
       <x:c r="D26" s="5" t="s">
-        <x:v>57</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E26" s="6" t="s">
-        <x:v>72</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F26" s="7"/>
       <x:c r="G26" s="8"/>
       <x:c r="H26" s="6"/>
       <x:c r="I26" s="7"/>
     </x:row>
-    <x:row r="27" spans="1:9" s="16" customFormat="1" ht="13.19999999999999928946">
-      <x:c r="A27" s="15" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="B27" s="13"/>
-      <x:c r="C27" s="13"/>
-      <x:c r="D27" s="13"/>
-      <x:c r="E27" s="13"/>
-      <x:c r="F27" s="13"/>
-      <x:c r="G27" s="13"/>
-      <x:c r="H27" s="13"/>
-      <x:c r="I27" s="14"/>
-    </x:row>
-    <x:row r="28" spans="1:9" s="16" customFormat="1" ht="13.19999999999999928946">
+    <x:row r="27" spans="1:9" s="12" customFormat="1" ht="13.19999999999999928946">
+      <x:c r="A27" s="19" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B27" s="17"/>
+      <x:c r="C27" s="17"/>
+      <x:c r="D27" s="17"/>
+      <x:c r="E27" s="17"/>
+      <x:c r="F27" s="17"/>
+      <x:c r="G27" s="17"/>
+      <x:c r="H27" s="17"/>
+      <x:c r="I27" s="18"/>
+    </x:row>
+    <x:row r="28" spans="1:9" s="12" customFormat="1" ht="13.19999999999999928946">
       <x:c r="A28" s="2"/>
       <x:c r="B28" s="3" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C28" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D28" s="5" t="s">
-        <x:v>28</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E28" s="6"/>
       <x:c r="F28" s="7"/>
@@ -1510,16 +1514,16 @@
       <x:c r="H28" s="6"/>
       <x:c r="I28" s="7"/>
     </x:row>
-    <x:row r="29" spans="1:9" s="16" customFormat="1" ht="13.19999999999999928946">
+    <x:row r="29" spans="1:9" s="12" customFormat="1" ht="13.19999999999999928946">
       <x:c r="A29" s="2"/>
       <x:c r="B29" s="3" t="s">
-        <x:v>27</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C29" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D29" s="5" t="s">
-        <x:v>60</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E29" s="6"/>
       <x:c r="F29" s="7"/>
@@ -1527,16 +1531,16 @@
       <x:c r="H29" s="6"/>
       <x:c r="I29" s="7"/>
     </x:row>
-    <x:row r="30" spans="1:9" s="16" customFormat="1" ht="13.19999999999999928946">
+    <x:row r="30" spans="1:9" s="12" customFormat="1" ht="13.19999999999999928946">
       <x:c r="A30" s="2"/>
       <x:c r="B30" s="3" t="s">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C30" s="4" t="s">
         <x:v>39</x:v>
       </x:c>
       <x:c r="D30" s="5" t="s">
-        <x:v>28</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E30" s="6"/>
       <x:c r="F30" s="7"/>
@@ -1544,16 +1548,16 @@
       <x:c r="H30" s="6"/>
       <x:c r="I30" s="7"/>
     </x:row>
-    <x:row r="31" spans="1:9" s="16" customFormat="1" ht="13.19999999999999928946">
+    <x:row r="31" spans="1:9" s="12" customFormat="1" ht="13.19999999999999928946">
       <x:c r="A31" s="2"/>
       <x:c r="B31" s="3" t="s">
-        <x:v>43</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C31" s="11" t="s">
-        <x:v>34</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="D31" s="5" t="s">
-        <x:v>60</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E31" s="6"/>
       <x:c r="F31" s="7"/>
@@ -1561,16 +1565,16 @@
       <x:c r="H31" s="6"/>
       <x:c r="I31" s="7"/>
     </x:row>
-    <x:row r="32" spans="1:9" s="16" customFormat="1" ht="13.19999999999999928946">
+    <x:row r="32" spans="1:9" s="12" customFormat="1" ht="13.19999999999999928946">
       <x:c r="A32" s="2"/>
       <x:c r="B32" s="3" t="s">
-        <x:v>48</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C32" s="10" t="s">
-        <x:v>54</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D32" s="5" t="s">
-        <x:v>60</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E32" s="6"/>
       <x:c r="F32" s="7"/>
@@ -1578,97 +1582,100 @@
       <x:c r="H32" s="6"/>
       <x:c r="I32" s="7"/>
     </x:row>
-    <x:row r="33" spans="1:9" s="17" customFormat="1" ht="13.55000000000000071054" customHeight="1">
-      <x:c r="A33" s="19"/>
+    <x:row r="33" spans="1:9" s="13" customFormat="1" ht="13.55000000000000071054" customHeight="1">
+      <x:c r="A33" s="15"/>
       <x:c r="B33" s="3" t="s">
-        <x:v>43</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C33" s="11" t="s">
-        <x:v>34</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="D33" s="5" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="E33" s="19"/>
-      <x:c r="F33" s="19"/>
-      <x:c r="G33" s="19"/>
-      <x:c r="H33" s="18"/>
-      <x:c r="I33" s="18"/>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E33" s="15"/>
+      <x:c r="F33" s="15"/>
+      <x:c r="G33" s="15"/>
+      <x:c r="H33" s="14"/>
+      <x:c r="I33" s="14"/>
     </x:row>
     <x:row r="34" spans="2:4" customHeight="1">
       <x:c r="B34" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="C34" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="C34" t="s">
-        <x:v>31</x:v>
-      </x:c>
       <x:c r="D34" t="s">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="2:4" customHeight="1">
       <x:c r="B35" t="s">
-        <x:v>63</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C35" t="s">
         <x:v>39</x:v>
       </x:c>
       <x:c r="D35" t="s">
-        <x:v>68</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="2:4" customHeight="1">
       <x:c r="B36" t="s">
-        <x:v>62</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C36" t="s">
-        <x:v>54</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D36" t="s">
-        <x:v>71</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="2:4" customHeight="1">
       <x:c r="B37" t="s">
-        <x:v>22</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C37" t="s">
         <x:v>39</x:v>
       </x:c>
       <x:c r="D37" t="s">
-        <x:v>66</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="2:4" customHeight="1">
       <x:c r="B38" t="s">
-        <x:v>3</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C38" t="s">
         <x:v>39</x:v>
       </x:c>
       <x:c r="D38" t="s">
-        <x:v>67</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:9" customHeight="1">
-      <x:c r="A39" s="21" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="B39" s="20"/>
-      <x:c r="C39" s="20"/>
-      <x:c r="D39" s="20"/>
-      <x:c r="E39" s="20"/>
-      <x:c r="F39" s="20"/>
-      <x:c r="G39" s="20"/>
-      <x:c r="H39" s="20"/>
-      <x:c r="I39" s="20"/>
-    </x:row>
-    <x:row r="40" spans="3:4" customHeight="1">
+      <x:c r="A39" s="20" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B39" s="21"/>
+      <x:c r="C39" s="21"/>
+      <x:c r="D39" s="21"/>
+      <x:c r="E39" s="21"/>
+      <x:c r="F39" s="21"/>
+      <x:c r="G39" s="21"/>
+      <x:c r="H39" s="21"/>
+      <x:c r="I39" s="21"/>
+    </x:row>
+    <x:row r="40" spans="3:5" customHeight="1">
       <x:c r="C40" t="s">
         <x:v>39</x:v>
       </x:c>
       <x:c r="D40" t="s">
-        <x:v>65</x:v>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E40" t="s">
+        <x:v>40</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1697,7 +1704,7 @@
       <x:formula>LEN(TRIM(B33))&gt;0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:pageMargins left="0.74805557727813720703" right="0.74805557727813720703" top="0.98430556058883666992" bottom="0.98430556058883666992" header="0.51180553436279296875" footer="0.51180553436279296875"/>
+  <x:pageMargins left="0.74805557727813720703" right="0.74805557727813720703" top="0.98430556058883666992" bottom="0.98430556058883666992" header="0.51152777671813964844" footer="0.51152777671813964844"/>
   <x:pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="0" fitToHeight="0" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" useFirstPageNumber="0" horizontalDpi="0" verticalDpi="0" copies="1"/>
 </x:worksheet>
 </file>
</xml_diff>